<commit_message>
feat: add Hospitals to Risk Dashboard EAD display
Updates:
- Regenerated risk.json with hospital damage data from updated Excel files
- Added 'hospitals' to DISPLAY_ASSET_KEYS (schools excluded - unreliable)
- Updated EadBarChart to include hospitals in Facilities group

Hospital Damage Examples (Present Breaches):
- 500yr: $9.1M total (Qambar Shahdadkot: $6.4M highest)
- 100yr: $3.8M total
- 25yr: $1.7M total
- 10yr: $517K total

Note: Schools remain excluded due to unreliable data source.
</commit_message>
<xml_diff>
--- a/risk/Risk_Analysis_T3_100yrs_Future_Breaches.xlsx
+++ b/risk/Risk_Analysis_T3_100yrs_Future_Breaches.xlsx
@@ -538,7 +538,7 @@
         <v>61800</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J4" t="n">
         <v>39</v>
@@ -576,7 +576,7 @@
         <v>53760</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J5" t="n">
         <v>25</v>
@@ -614,7 +614,7 @@
         <v>45930</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J6" t="n">
         <v>13</v>
@@ -652,7 +652,7 @@
         <v>42690</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J7" t="n">
         <v>11</v>
@@ -690,7 +690,7 @@
         <v>27600</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J8" t="n">
         <v>10</v>
@@ -728,7 +728,7 @@
         <v>9450</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" t="n">
         <v>4</v>
@@ -804,7 +804,7 @@
         <v>4680</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J11" t="n">
         <v>3</v>
@@ -918,7 +918,7 @@
         <v>720</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -1660,7 +1660,7 @@
         <v>3690</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -1736,7 +1736,7 @@
         <v>4260</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J11" t="n">
         <v>1</v>
@@ -1850,7 +1850,7 @@
         <v>720</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -2592,7 +2592,7 @@
         <v>3690</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>0.88</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -2668,7 +2668,7 @@
         <v>4260</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J11" t="n">
         <v>1</v>
@@ -2782,7 +2782,7 @@
         <v>720</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -3524,7 +3524,7 @@
         <v>1020838.5</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>337330.4</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -3600,7 +3600,7 @@
         <v>1178529</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>766660</v>
       </c>
       <c r="J11" t="n">
         <v>58333</v>
@@ -3714,7 +3714,7 @@
         <v>199188</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>383330</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -9858,7 +9858,7 @@
         <v>7110</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J4" t="n">
         <v>9</v>
@@ -9896,7 +9896,7 @@
         <v>6210</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J5" t="n">
         <v>10</v>
@@ -9934,7 +9934,7 @@
         <v>7710</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J6" t="n">
         <v>6</v>
@@ -9972,7 +9972,7 @@
         <v>11820</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J7" t="n">
         <v>1</v>
@@ -10010,7 +10010,7 @@
         <v>2610</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J8" t="n">
         <v>2</v>
@@ -10124,7 +10124,7 @@
         <v>30</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -10828,7 +10828,7 @@
         <v>19353.6</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="J5" t="n">
         <v>7.5</v>
@@ -10866,7 +10866,7 @@
         <v>26180.1</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>0.35</v>
       </c>
       <c r="J6" t="n">
         <v>6.5</v>
@@ -10904,7 +10904,7 @@
         <v>31163.7</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="J7" t="n">
         <v>7.7</v>
@@ -10942,7 +10942,7 @@
         <v>23460</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>2.16</v>
       </c>
       <c r="J8" t="n">
         <v>8.5</v>
@@ -10980,7 +10980,7 @@
         <v>9450</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>0.88</v>
       </c>
       <c r="J9" t="n">
         <v>3.8</v>
@@ -11056,7 +11056,7 @@
         <v>4680</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J11" t="n">
         <v>3</v>
@@ -11170,7 +11170,7 @@
         <v>720</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -11760,7 +11760,7 @@
         <v>2235.6</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="J5" t="n">
         <v>3</v>
@@ -11798,7 +11798,7 @@
         <v>4394.7</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>0.35</v>
       </c>
       <c r="J6" t="n">
         <v>3</v>
@@ -11836,7 +11836,7 @@
         <v>8628.6</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="J7" t="n">
         <v>0.7</v>
@@ -11874,7 +11874,7 @@
         <v>2218.5</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>1.44</v>
       </c>
       <c r="J8" t="n">
         <v>1.7</v>
@@ -11988,7 +11988,7 @@
         <v>30</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -12692,7 +12692,7 @@
         <v>618478.74</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>229998</v>
       </c>
       <c r="J5" t="n">
         <v>174999</v>
@@ -12730,7 +12730,7 @@
         <v>1215793.75</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>134165.5</v>
       </c>
       <c r="J6" t="n">
         <v>174999</v>
@@ -12768,7 +12768,7 @@
         <v>2387102.19</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>421663</v>
       </c>
       <c r="J7" t="n">
         <v>40833.1</v>
@@ -12806,7 +12806,7 @@
         <v>613748.02</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>551995.2</v>
       </c>
       <c r="J8" t="n">
         <v>99166.10000000001</v>
@@ -12920,7 +12920,7 @@
         <v>8299.5</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>383330</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -13586,7 +13586,7 @@
         <v>13620</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
         <v>4</v>
@@ -16420,7 +16420,7 @@
         <v>5354173.44</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>287497.5</v>
       </c>
       <c r="J5" t="n">
         <v>437497.5</v>
@@ -16458,7 +16458,7 @@
         <v>7242724.66</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>134165.5</v>
       </c>
       <c r="J6" t="n">
         <v>379164.5</v>
@@ -16496,7 +16496,7 @@
         <v>8621437.6</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>421663</v>
       </c>
       <c r="J7" t="n">
         <v>449164.1</v>
@@ -16534,7 +16534,7 @@
         <v>6490209</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>827992.8</v>
       </c>
       <c r="J8" t="n">
         <v>495830.5</v>
@@ -16572,7 +16572,7 @@
         <v>2614342.5</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>337330.4</v>
       </c>
       <c r="J9" t="n">
         <v>221665.4</v>
@@ -16648,7 +16648,7 @@
         <v>1294722</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>1149990</v>
       </c>
       <c r="J11" t="n">
         <v>174999</v>
@@ -16762,7 +16762,7 @@
         <v>199188</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>383330</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -17314,7 +17314,7 @@
         <v>2880</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -17466,7 +17466,7 @@
         <v>20100</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J8" t="n">
         <v>7</v>
@@ -18398,7 +18398,7 @@
         <v>17085</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>0.72</v>
       </c>
       <c r="J8" t="n">
         <v>5.95</v>
@@ -19330,7 +19330,7 @@
         <v>4726565.25</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>275997.6</v>
       </c>
       <c r="J8" t="n">
         <v>347081.35</v>
@@ -20110,7 +20110,7 @@
         <v>17430</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
         <v>14</v>
@@ -20148,7 +20148,7 @@
         <v>22620</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
         <v>7</v>
@@ -21080,7 +21080,7 @@
         <v>8143.2</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="J5" t="n">
         <v>2.1</v>
@@ -22012,7 +22012,7 @@
         <v>2252816.28</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>57499.5</v>
       </c>
       <c r="J5" t="n">
         <v>122499.3</v>

</xml_diff>

<commit_message>
feat: add Schools to Risk Dashboard EAD display
Schools data has been added to all 42 risk Excel files and is now
included in risk.json. Schools contribute ~10x more damage than
hospitals and is now visible in the EAD view.

Schools Damage Examples (Present Breaches):
- 25yr: $27.1M vs Hospitals $1.7M
- 100yr: $50.1M vs Hospitals $3.8M
- 500yr: $85.0M vs Hospitals $9.1M

Changes:
- Regenerated risk.json with schools data
- Added 'schools' to DISPLAY_ASSET_KEYS
- Updated EadBarChart facilities group: [hospitals, bhu, schools]
</commit_message>
<xml_diff>
--- a/risk/Risk_Analysis_T3_100yrs_Future_Breaches.xlsx
+++ b/risk/Risk_Analysis_T3_100yrs_Future_Breaches.xlsx
@@ -544,7 +544,7 @@
         <v>39</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>1128</v>
       </c>
       <c r="L4" t="n">
         <v>1422210</v>
@@ -582,7 +582,7 @@
         <v>25</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>621</v>
       </c>
       <c r="L5" t="n">
         <v>890580</v>
@@ -620,7 +620,7 @@
         <v>13</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>431</v>
       </c>
       <c r="L6" t="n">
         <v>576900</v>
@@ -658,7 +658,7 @@
         <v>11</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>448</v>
       </c>
       <c r="L7" t="n">
         <v>534450</v>
@@ -696,7 +696,7 @@
         <v>10</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>355</v>
       </c>
       <c r="L8" t="n">
         <v>442920</v>
@@ -734,7 +734,7 @@
         <v>4</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>342</v>
       </c>
       <c r="L9" t="n">
         <v>377130</v>
@@ -772,7 +772,7 @@
         <v>11</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>255</v>
       </c>
       <c r="L10" t="n">
         <v>299550</v>
@@ -810,7 +810,7 @@
         <v>3</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>173</v>
       </c>
       <c r="L11" t="n">
         <v>187590</v>
@@ -848,7 +848,7 @@
         <v>2</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>114</v>
       </c>
       <c r="L12" t="n">
         <v>151800</v>
@@ -886,7 +886,7 @@
         <v>3</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="L13" t="n">
         <v>102240</v>
@@ -924,7 +924,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="L14" t="n">
         <v>43560</v>
@@ -962,7 +962,7 @@
         <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="L15" t="n">
         <v>18390</v>
@@ -1000,7 +1000,7 @@
         <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L16" t="n">
         <v>8700</v>
@@ -1038,7 +1038,7 @@
         <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L17" t="n">
         <v>2460</v>
@@ -1076,7 +1076,7 @@
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L18" t="n">
         <v>4620</v>
@@ -1476,7 +1476,7 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="L4" t="n">
         <v>17160</v>
@@ -1514,7 +1514,7 @@
         <v>3</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L5" t="n">
         <v>20430</v>
@@ -1552,7 +1552,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="L6" t="n">
         <v>21240</v>
@@ -1590,7 +1590,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="L7" t="n">
         <v>26430</v>
@@ -1628,7 +1628,7 @@
         <v>1</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="L8" t="n">
         <v>36630</v>
@@ -1666,7 +1666,7 @@
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="L9" t="n">
         <v>45870</v>
@@ -1704,7 +1704,7 @@
         <v>5</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="L10" t="n">
         <v>43620</v>
@@ -1742,7 +1742,7 @@
         <v>1</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="L11" t="n">
         <v>53730</v>
@@ -1780,7 +1780,7 @@
         <v>1</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="L12" t="n">
         <v>91590</v>
@@ -1818,7 +1818,7 @@
         <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="L13" t="n">
         <v>71640</v>
@@ -1856,7 +1856,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="L14" t="n">
         <v>33870</v>
@@ -1894,7 +1894,7 @@
         <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="L15" t="n">
         <v>14460</v>
@@ -1932,7 +1932,7 @@
         <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L16" t="n">
         <v>7500</v>
@@ -1970,7 +1970,7 @@
         <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L17" t="n">
         <v>1860</v>
@@ -2008,7 +2008,7 @@
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L18" t="n">
         <v>3810</v>
@@ -2446,7 +2446,7 @@
         <v>0.9</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>2.94</v>
       </c>
       <c r="L5" t="n">
         <v>4290.3</v>
@@ -2484,7 +2484,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="L6" t="n">
         <v>7858.8</v>
@@ -2522,7 +2522,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>16.4</v>
       </c>
       <c r="L7" t="n">
         <v>15858</v>
@@ -2560,7 +2560,7 @@
         <v>0.85</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>16.2</v>
       </c>
       <c r="L8" t="n">
         <v>26007.3</v>
@@ -2598,7 +2598,7 @@
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="L9" t="n">
         <v>37154.7</v>
@@ -2636,7 +2636,7 @@
         <v>5</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="L10" t="n">
         <v>38821.8</v>
@@ -2674,7 +2674,7 @@
         <v>1</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="L11" t="n">
         <v>53730</v>
@@ -2712,7 +2712,7 @@
         <v>1</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="L12" t="n">
         <v>91590</v>
@@ -2750,7 +2750,7 @@
         <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="L13" t="n">
         <v>71640</v>
@@ -2788,7 +2788,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="L14" t="n">
         <v>33870</v>
@@ -2826,7 +2826,7 @@
         <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="L15" t="n">
         <v>14460</v>
@@ -2864,7 +2864,7 @@
         <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L16" t="n">
         <v>7500</v>
@@ -2902,7 +2902,7 @@
         <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L17" t="n">
         <v>1860</v>
@@ -2940,7 +2940,7 @@
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L18" t="n">
         <v>3810</v>
@@ -3378,7 +3378,7 @@
         <v>52499.7</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>62721.96</v>
       </c>
       <c r="L5" t="n">
         <v>40414.63</v>
@@ -3416,7 +3416,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>277342</v>
       </c>
       <c r="L6" t="n">
         <v>74029.89999999999</v>
@@ -3454,7 +3454,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>349877.6</v>
       </c>
       <c r="L7" t="n">
         <v>149382.36</v>
@@ -3492,7 +3492,7 @@
         <v>49583.05</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>345610.8</v>
       </c>
       <c r="L8" t="n">
         <v>244988.77</v>
@@ -3530,7 +3530,7 @@
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>597352</v>
       </c>
       <c r="L9" t="n">
         <v>349997.27</v>
@@ -3568,7 +3568,7 @@
         <v>291665</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>362678</v>
       </c>
       <c r="L10" t="n">
         <v>365701.36</v>
@@ -3606,7 +3606,7 @@
         <v>58333</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>618686</v>
       </c>
       <c r="L11" t="n">
         <v>506136.6</v>
@@ -3644,7 +3644,7 @@
         <v>58333</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>853360</v>
       </c>
       <c r="L12" t="n">
         <v>862777.8</v>
@@ -3682,7 +3682,7 @@
         <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>661354</v>
       </c>
       <c r="L13" t="n">
         <v>674848.8</v>
@@ -3720,7 +3720,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>490682</v>
       </c>
       <c r="L14" t="n">
         <v>319055.4</v>
@@ -3758,7 +3758,7 @@
         <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>192006</v>
       </c>
       <c r="L15" t="n">
         <v>136213.2</v>
@@ -3796,7 +3796,7 @@
         <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>64002</v>
       </c>
       <c r="L16" t="n">
         <v>70650</v>
@@ -3834,7 +3834,7 @@
         <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>21334</v>
       </c>
       <c r="L17" t="n">
         <v>17521.2</v>
@@ -3872,7 +3872,7 @@
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>21334</v>
       </c>
       <c r="L18" t="n">
         <v>35890.2</v>
@@ -4272,7 +4272,7 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="L4" t="n">
         <v>145950</v>
@@ -4310,7 +4310,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="L5" t="n">
         <v>57990</v>
@@ -4348,7 +4348,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L6" t="n">
         <v>11280</v>
@@ -4386,7 +4386,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L7" t="n">
         <v>3090</v>
@@ -5242,7 +5242,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>12.18</v>
       </c>
       <c r="L5" t="n">
         <v>12177.9</v>
@@ -5280,7 +5280,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>0.65</v>
       </c>
       <c r="L6" t="n">
         <v>4173.6</v>
@@ -5318,7 +5318,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>0.82</v>
       </c>
       <c r="L7" t="n">
         <v>1854</v>
@@ -6174,7 +6174,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>259848.12</v>
       </c>
       <c r="L5" t="n">
         <v>114715.82</v>
@@ -6212,7 +6212,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>13867.1</v>
       </c>
       <c r="L6" t="n">
         <v>39315.31</v>
@@ -6250,7 +6250,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>17493.88</v>
       </c>
       <c r="L7" t="n">
         <v>17464.68</v>
@@ -7068,7 +7068,7 @@
         <v>10</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>175</v>
       </c>
       <c r="L4" t="n">
         <v>138090</v>
@@ -7106,7 +7106,7 @@
         <v>1</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="L5" t="n">
         <v>48120</v>
@@ -7144,7 +7144,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="L6" t="n">
         <v>13800</v>
@@ -7182,7 +7182,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L7" t="n">
         <v>3780</v>
@@ -7220,7 +7220,7 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L8" t="n">
         <v>2040</v>
@@ -8038,7 +8038,7 @@
         <v>0.3</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>20.16</v>
       </c>
       <c r="L5" t="n">
         <v>10105.2</v>
@@ -8076,7 +8076,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>5.85</v>
       </c>
       <c r="L6" t="n">
         <v>5106</v>
@@ -8114,7 +8114,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>1.64</v>
       </c>
       <c r="L7" t="n">
         <v>2268</v>
@@ -8152,7 +8152,7 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>1.8</v>
       </c>
       <c r="L8" t="n">
         <v>1448.4</v>
@@ -8970,7 +8970,7 @@
         <v>17499.9</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>430093.44</v>
       </c>
       <c r="L5" t="n">
         <v>95190.98</v>
@@ -9008,7 +9008,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>124803.9</v>
       </c>
       <c r="L6" t="n">
         <v>48098.52</v>
@@ -9046,7 +9046,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>34987.76</v>
       </c>
       <c r="L7" t="n">
         <v>21364.56</v>
@@ -9084,7 +9084,7 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>38401.2</v>
       </c>
       <c r="L8" t="n">
         <v>13643.93</v>
@@ -9864,7 +9864,7 @@
         <v>9</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>229</v>
       </c>
       <c r="L4" t="n">
         <v>172020</v>
@@ -9902,7 +9902,7 @@
         <v>10</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>161</v>
       </c>
       <c r="L5" t="n">
         <v>162150</v>
@@ -9940,7 +9940,7 @@
         <v>6</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>151</v>
       </c>
       <c r="L6" t="n">
         <v>156240</v>
@@ -9978,7 +9978,7 @@
         <v>1</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>204</v>
       </c>
       <c r="L7" t="n">
         <v>202350</v>
@@ -10016,7 +10016,7 @@
         <v>2</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>125</v>
       </c>
       <c r="L8" t="n">
         <v>127200</v>
@@ -10054,7 +10054,7 @@
         <v>1</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>92</v>
       </c>
       <c r="L9" t="n">
         <v>74580</v>
@@ -10092,7 +10092,7 @@
         <v>2</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="L10" t="n">
         <v>39240</v>
@@ -10130,7 +10130,7 @@
         <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L11" t="n">
         <v>10200</v>
@@ -10168,7 +10168,7 @@
         <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L12" t="n">
         <v>4740</v>
@@ -10396,7 +10396,7 @@
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L18" t="n">
         <v>600</v>
@@ -10834,7 +10834,7 @@
         <v>7.5</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>260.82</v>
       </c>
       <c r="L5" t="n">
         <v>187021.8</v>
@@ -10872,7 +10872,7 @@
         <v>6.5</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>280.15</v>
       </c>
       <c r="L6" t="n">
         <v>213453</v>
@@ -10910,7 +10910,7 @@
         <v>7.7</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>367.36</v>
       </c>
       <c r="L7" t="n">
         <v>320670</v>
@@ -10948,7 +10948,7 @@
         <v>8.5</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>319.5</v>
       </c>
       <c r="L8" t="n">
         <v>314473.2</v>
@@ -10986,7 +10986,7 @@
         <v>3.8</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>342</v>
       </c>
       <c r="L9" t="n">
         <v>305475.3</v>
@@ -11024,7 +11024,7 @@
         <v>11</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>255</v>
       </c>
       <c r="L10" t="n">
         <v>266599.5</v>
@@ -11062,7 +11062,7 @@
         <v>3</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>173</v>
       </c>
       <c r="L11" t="n">
         <v>187590</v>
@@ -11100,7 +11100,7 @@
         <v>2</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>114</v>
       </c>
       <c r="L12" t="n">
         <v>151800</v>
@@ -11138,7 +11138,7 @@
         <v>3</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="L13" t="n">
         <v>102240</v>
@@ -11176,7 +11176,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="L14" t="n">
         <v>43560</v>
@@ -11214,7 +11214,7 @@
         <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="L15" t="n">
         <v>18390</v>
@@ -11252,7 +11252,7 @@
         <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L16" t="n">
         <v>8700</v>
@@ -11290,7 +11290,7 @@
         <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L17" t="n">
         <v>2460</v>
@@ -11328,7 +11328,7 @@
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L18" t="n">
         <v>4620</v>
@@ -11766,7 +11766,7 @@
         <v>3</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>67.62</v>
       </c>
       <c r="L5" t="n">
         <v>34051.5</v>
@@ -11804,7 +11804,7 @@
         <v>3</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>98.15000000000001</v>
       </c>
       <c r="L6" t="n">
         <v>57808.8</v>
@@ -11842,7 +11842,7 @@
         <v>0.7</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>167.28</v>
       </c>
       <c r="L7" t="n">
         <v>121410</v>
@@ -11880,7 +11880,7 @@
         <v>1.7</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>112.5</v>
       </c>
       <c r="L8" t="n">
         <v>90312</v>
@@ -11918,7 +11918,7 @@
         <v>0.95</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>92</v>
       </c>
       <c r="L9" t="n">
         <v>60409.8</v>
@@ -11956,7 +11956,7 @@
         <v>2</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="L10" t="n">
         <v>34923.6</v>
@@ -11994,7 +11994,7 @@
         <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L11" t="n">
         <v>10200</v>
@@ -12032,7 +12032,7 @@
         <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L12" t="n">
         <v>4740</v>
@@ -12260,7 +12260,7 @@
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L18" t="n">
         <v>600</v>
@@ -12698,7 +12698,7 @@
         <v>174999</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>1442605.08</v>
       </c>
       <c r="L5" t="n">
         <v>320765.13</v>
@@ -12736,7 +12736,7 @@
         <v>174999</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>2093932.1</v>
       </c>
       <c r="L6" t="n">
         <v>544558.9</v>
@@ -12774,7 +12774,7 @@
         <v>40833.1</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>3568751.52</v>
       </c>
       <c r="L7" t="n">
         <v>1143682.2</v>
@@ -12812,7 +12812,7 @@
         <v>99166.10000000001</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>2400075</v>
       </c>
       <c r="L8" t="n">
         <v>850739.04</v>
@@ -12850,7 +12850,7 @@
         <v>55416.35</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>1962728</v>
       </c>
       <c r="L9" t="n">
         <v>569060.3199999999</v>
@@ -12888,7 +12888,7 @@
         <v>116666</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>960030</v>
       </c>
       <c r="L10" t="n">
         <v>328980.31</v>
@@ -12926,7 +12926,7 @@
         <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>106670</v>
       </c>
       <c r="L11" t="n">
         <v>96084</v>
@@ -12964,7 +12964,7 @@
         <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>42668</v>
       </c>
       <c r="L12" t="n">
         <v>44650.8</v>
@@ -13192,7 +13192,7 @@
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>21334</v>
       </c>
       <c r="L18" t="n">
         <v>5652</v>
@@ -13592,7 +13592,7 @@
         <v>4</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>118</v>
       </c>
       <c r="L4" t="n">
         <v>343380</v>
@@ -13630,7 +13630,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="L5" t="n">
         <v>110970</v>
@@ -14562,7 +14562,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>13.44</v>
       </c>
       <c r="L5" t="n">
         <v>23303.7</v>
@@ -15494,7 +15494,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>286728.96</v>
       </c>
       <c r="L5" t="n">
         <v>219520.85</v>
@@ -16426,7 +16426,7 @@
         <v>437497.5</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>5564333.88</v>
       </c>
       <c r="L5" t="n">
         <v>1761745.36</v>
@@ -16464,7 +16464,7 @@
         <v>379164.5</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>5976720.1</v>
       </c>
       <c r="L6" t="n">
         <v>2010727.26</v>
@@ -16502,7 +16502,7 @@
         <v>449164.1</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>7837258.24</v>
       </c>
       <c r="L7" t="n">
         <v>3020711.4</v>
@@ -16540,7 +16540,7 @@
         <v>495830.5</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>6816213</v>
       </c>
       <c r="L8" t="n">
         <v>2962337.54</v>
@@ -16578,7 +16578,7 @@
         <v>221665.4</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>7296228</v>
       </c>
       <c r="L9" t="n">
         <v>2877577.33</v>
@@ -16616,7 +16616,7 @@
         <v>641663</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>5440170</v>
       </c>
       <c r="L10" t="n">
         <v>2511367.29</v>
@@ -16654,7 +16654,7 @@
         <v>174999</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>3690782</v>
       </c>
       <c r="L11" t="n">
         <v>1767097.8</v>
@@ -16692,7 +16692,7 @@
         <v>116666</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>2432076</v>
       </c>
       <c r="L12" t="n">
         <v>1429956</v>
@@ -16730,7 +16730,7 @@
         <v>174999</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>1194704</v>
       </c>
       <c r="L13" t="n">
         <v>963100.8</v>
@@ -16768,7 +16768,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>704022</v>
       </c>
       <c r="L14" t="n">
         <v>410335.2</v>
@@ -16806,7 +16806,7 @@
         <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>192006</v>
       </c>
       <c r="L15" t="n">
         <v>173233.8</v>
@@ -16844,7 +16844,7 @@
         <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>85336</v>
       </c>
       <c r="L16" t="n">
         <v>81954</v>
@@ -16882,7 +16882,7 @@
         <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>42668</v>
       </c>
       <c r="L17" t="n">
         <v>23173.2</v>
@@ -16920,7 +16920,7 @@
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>42668</v>
       </c>
       <c r="L18" t="n">
         <v>43520.4</v>
@@ -17320,7 +17320,7 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>140</v>
       </c>
       <c r="L4" t="n">
         <v>138840</v>
@@ -17358,7 +17358,7 @@
         <v>2</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>152</v>
       </c>
       <c r="L5" t="n">
         <v>166950</v>
@@ -17396,7 +17396,7 @@
         <v>4</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>141</v>
       </c>
       <c r="L6" t="n">
         <v>169050</v>
@@ -17434,7 +17434,7 @@
         <v>7</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>145</v>
       </c>
       <c r="L7" t="n">
         <v>180720</v>
@@ -17472,7 +17472,7 @@
         <v>7</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>201</v>
       </c>
       <c r="L8" t="n">
         <v>237450</v>
@@ -17510,7 +17510,7 @@
         <v>3</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>219</v>
       </c>
       <c r="L9" t="n">
         <v>239250</v>
@@ -17548,7 +17548,7 @@
         <v>4</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>192</v>
       </c>
       <c r="L10" t="n">
         <v>208230</v>
@@ -17586,7 +17586,7 @@
         <v>2</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>139</v>
       </c>
       <c r="L11" t="n">
         <v>121290</v>
@@ -17624,7 +17624,7 @@
         <v>1</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="L12" t="n">
         <v>54630</v>
@@ -17662,7 +17662,7 @@
         <v>3</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="L13" t="n">
         <v>27150</v>
@@ -17700,7 +17700,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L14" t="n">
         <v>8100</v>
@@ -17776,7 +17776,7 @@
         <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L16" t="n">
         <v>960</v>
@@ -17814,7 +17814,7 @@
         <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L17" t="n">
         <v>210</v>
@@ -18290,7 +18290,7 @@
         <v>0.6</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>63.84</v>
       </c>
       <c r="L5" t="n">
         <v>35059.5</v>
@@ -18328,7 +18328,7 @@
         <v>2</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>91.65000000000001</v>
       </c>
       <c r="L6" t="n">
         <v>62548.5</v>
@@ -18366,7 +18366,7 @@
         <v>4.9</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>118.9</v>
       </c>
       <c r="L7" t="n">
         <v>108432</v>
@@ -18404,7 +18404,7 @@
         <v>5.95</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>180.9</v>
       </c>
       <c r="L8" t="n">
         <v>168589.5</v>
@@ -18442,7 +18442,7 @@
         <v>2.85</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>219</v>
       </c>
       <c r="L9" t="n">
         <v>193792.5</v>
@@ -18480,7 +18480,7 @@
         <v>4</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>192</v>
       </c>
       <c r="L10" t="n">
         <v>185324.7</v>
@@ -18518,7 +18518,7 @@
         <v>2</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>139</v>
       </c>
       <c r="L11" t="n">
         <v>121290</v>
@@ -18556,7 +18556,7 @@
         <v>1</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="L12" t="n">
         <v>54630</v>
@@ -18594,7 +18594,7 @@
         <v>3</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="L13" t="n">
         <v>27150</v>
@@ -18632,7 +18632,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="L14" t="n">
         <v>8100</v>
@@ -18708,7 +18708,7 @@
         <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L16" t="n">
         <v>960</v>
@@ -18746,7 +18746,7 @@
         <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L17" t="n">
         <v>210</v>
@@ -19222,7 +19222,7 @@
         <v>34999.8</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>1361962.56</v>
       </c>
       <c r="L5" t="n">
         <v>330260.49</v>
@@ -19260,7 +19260,7 @@
         <v>116666</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>1955261.1</v>
       </c>
       <c r="L6" t="n">
         <v>589206.87</v>
@@ -19298,7 +19298,7 @@
         <v>285831.7</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>2536612.6</v>
       </c>
       <c r="L7" t="n">
         <v>1021429.44</v>
@@ -19336,7 +19336,7 @@
         <v>347081.35</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>3859320.6</v>
       </c>
       <c r="L8" t="n">
         <v>1588113.09</v>
@@ -19374,7 +19374,7 @@
         <v>166249.05</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>4672146</v>
       </c>
       <c r="L9" t="n">
         <v>1825525.35</v>
@@ -19412,7 +19412,7 @@
         <v>233332</v>
       </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>4096128</v>
       </c>
       <c r="L10" t="n">
         <v>1745758.67</v>
@@ -19450,7 +19450,7 @@
         <v>116666</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>2965426</v>
       </c>
       <c r="L11" t="n">
         <v>1142551.8</v>
@@ -19488,7 +19488,7 @@
         <v>58333</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>1536048</v>
       </c>
       <c r="L12" t="n">
         <v>514614.6</v>
@@ -19526,7 +19526,7 @@
         <v>174999</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>512016</v>
       </c>
       <c r="L13" t="n">
         <v>255753</v>
@@ -19564,7 +19564,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>213340</v>
       </c>
       <c r="L14" t="n">
         <v>76302</v>
@@ -19640,7 +19640,7 @@
         <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>21334</v>
       </c>
       <c r="L16" t="n">
         <v>9043.200000000001</v>
@@ -19678,7 +19678,7 @@
         <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>21334</v>
       </c>
       <c r="L17" t="n">
         <v>1978.2</v>
@@ -20116,7 +20116,7 @@
         <v>14</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>387</v>
       </c>
       <c r="L4" t="n">
         <v>408330</v>
@@ -20154,7 +20154,7 @@
         <v>7</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>191</v>
       </c>
       <c r="L5" t="n">
         <v>262830</v>
@@ -20192,7 +20192,7 @@
         <v>3</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>108</v>
       </c>
       <c r="L6" t="n">
         <v>134520</v>
@@ -20230,7 +20230,7 @@
         <v>3</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>74</v>
       </c>
       <c r="L7" t="n">
         <v>79440</v>
@@ -20268,7 +20268,7 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="L8" t="n">
         <v>21840</v>
@@ -21086,7 +21086,7 @@
         <v>2.1</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>80.22</v>
       </c>
       <c r="L5" t="n">
         <v>55194.3</v>
@@ -21124,7 +21124,7 @@
         <v>1.5</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>70.2</v>
       </c>
       <c r="L6" t="n">
         <v>49772.4</v>
@@ -21162,7 +21162,7 @@
         <v>2.1</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>60.68</v>
       </c>
       <c r="L7" t="n">
         <v>47664</v>
@@ -21200,7 +21200,7 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>8.1</v>
       </c>
       <c r="L8" t="n">
         <v>15506.4</v>
@@ -22018,7 +22018,7 @@
         <v>122499.3</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>1711413.48</v>
       </c>
       <c r="L5" t="n">
         <v>519930.31</v>
@@ -22056,7 +22056,7 @@
         <v>87499.5</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>1497646.8</v>
       </c>
       <c r="L6" t="n">
         <v>468856.01</v>
@@ -22094,7 +22094,7 @@
         <v>122499.3</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>1294547.12</v>
       </c>
       <c r="L7" t="n">
         <v>448994.88</v>
@@ -22132,7 +22132,7 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>172805.4</v>
       </c>
       <c r="L8" t="n">
         <v>146070.29</v>

</xml_diff>

<commit_message>
feat: update risk data with corrected Schools values
- Regenerated risk.json from updated Excel files
- Schools asset values reduced by ~70-75% across all 42 scenarios
- All other 11 assets unchanged (crop, buildings, telecom, electric, railways, hospitals, BHU, roads, hydraulic)
- Updated 42 Risk Analysis Excel files in risk/ folder
- Build: TypeScript check passed, Vite build successful

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/risk/Risk_Analysis_T3_100yrs_Future_Breaches.xlsx
+++ b/risk/Risk_Analysis_T3_100yrs_Future_Breaches.xlsx
@@ -549,7 +549,7 @@
         <v>39</v>
       </c>
       <c r="K4" t="n">
-        <v>1109</v>
+        <v>433</v>
       </c>
       <c r="L4" t="n">
         <v>1418940</v>
@@ -590,7 +590,7 @@
         <v>25</v>
       </c>
       <c r="K5" t="n">
-        <v>607</v>
+        <v>262</v>
       </c>
       <c r="L5" t="n">
         <v>888630</v>
@@ -631,7 +631,7 @@
         <v>13</v>
       </c>
       <c r="K6" t="n">
-        <v>426</v>
+        <v>165</v>
       </c>
       <c r="L6" t="n">
         <v>575160</v>
@@ -672,7 +672,7 @@
         <v>11</v>
       </c>
       <c r="K7" t="n">
-        <v>447</v>
+        <v>152</v>
       </c>
       <c r="L7" t="n">
         <v>533400</v>
@@ -713,7 +713,7 @@
         <v>10</v>
       </c>
       <c r="K8" t="n">
-        <v>355</v>
+        <v>102</v>
       </c>
       <c r="L8" t="n">
         <v>442200</v>
@@ -754,7 +754,7 @@
         <v>4</v>
       </c>
       <c r="K9" t="n">
-        <v>342</v>
+        <v>110</v>
       </c>
       <c r="L9" t="n">
         <v>376770</v>
@@ -795,7 +795,7 @@
         <v>11</v>
       </c>
       <c r="K10" t="n">
-        <v>255</v>
+        <v>59</v>
       </c>
       <c r="L10" t="n">
         <v>299460</v>
@@ -836,7 +836,7 @@
         <v>3</v>
       </c>
       <c r="K11" t="n">
-        <v>173</v>
+        <v>35</v>
       </c>
       <c r="L11" t="n">
         <v>187320</v>
@@ -877,7 +877,7 @@
         <v>2</v>
       </c>
       <c r="K12" t="n">
-        <v>114</v>
+        <v>17</v>
       </c>
       <c r="L12" t="n">
         <v>151590</v>
@@ -918,7 +918,7 @@
         <v>3</v>
       </c>
       <c r="K13" t="n">
-        <v>56</v>
+        <v>6</v>
       </c>
       <c r="L13" t="n">
         <v>102240</v>
@@ -959,7 +959,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="L14" t="n">
         <v>43560</v>
@@ -1000,7 +1000,7 @@
         <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L15" t="n">
         <v>18390</v>
@@ -1041,7 +1041,7 @@
         <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
         <v>8700</v>
@@ -1082,7 +1082,7 @@
         <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L17" t="n">
         <v>2460</v>
@@ -1123,7 +1123,7 @@
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
         <v>4620</v>
@@ -1553,7 +1553,7 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="L4" t="n">
         <v>17280</v>
@@ -1594,7 +1594,7 @@
         <v>3</v>
       </c>
       <c r="K5" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L5" t="n">
         <v>20400</v>
@@ -1635,7 +1635,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="L6" t="n">
         <v>21300</v>
@@ -1676,7 +1676,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="L7" t="n">
         <v>26490</v>
@@ -1717,7 +1717,7 @@
         <v>1</v>
       </c>
       <c r="K8" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="L8" t="n">
         <v>36840</v>
@@ -1758,7 +1758,7 @@
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="L9" t="n">
         <v>46050</v>
@@ -1799,7 +1799,7 @@
         <v>5</v>
       </c>
       <c r="K10" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="L10" t="n">
         <v>43650</v>
@@ -1840,7 +1840,7 @@
         <v>1</v>
       </c>
       <c r="K11" t="n">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="L11" t="n">
         <v>53910</v>
@@ -1881,7 +1881,7 @@
         <v>1</v>
       </c>
       <c r="K12" t="n">
-        <v>40</v>
+        <v>6</v>
       </c>
       <c r="L12" t="n">
         <v>91770</v>
@@ -1922,7 +1922,7 @@
         <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>31</v>
+        <v>5</v>
       </c>
       <c r="L13" t="n">
         <v>71700</v>
@@ -1963,7 +1963,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="L14" t="n">
         <v>33900</v>
@@ -2004,7 +2004,7 @@
         <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L15" t="n">
         <v>14520</v>
@@ -2045,7 +2045,7 @@
         <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
         <v>7500</v>
@@ -2086,7 +2086,7 @@
         <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L17" t="n">
         <v>1860</v>
@@ -2127,7 +2127,7 @@
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
         <v>3810</v>
@@ -2598,7 +2598,7 @@
         <v>0.9</v>
       </c>
       <c r="K5" t="n">
-        <v>1.99</v>
+        <v>0.99</v>
       </c>
       <c r="L5" t="n">
         <v>4284</v>
@@ -2639,7 +2639,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>10.14</v>
+        <v>4.56</v>
       </c>
       <c r="L6" t="n">
         <v>7881</v>
@@ -2680,7 +2680,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>12.76</v>
+        <v>6.38</v>
       </c>
       <c r="L7" t="n">
         <v>15894</v>
@@ -2721,7 +2721,7 @@
         <v>0.85</v>
       </c>
       <c r="K8" t="n">
-        <v>13.25</v>
+        <v>8.1</v>
       </c>
       <c r="L8" t="n">
         <v>26156.4</v>
@@ -2762,7 +2762,7 @@
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>22.48</v>
+        <v>8.029999999999999</v>
       </c>
       <c r="L9" t="n">
         <v>37300.5</v>
@@ -2803,7 +2803,7 @@
         <v>5</v>
       </c>
       <c r="K10" t="n">
-        <v>14.79</v>
+        <v>1.74</v>
       </c>
       <c r="L10" t="n">
         <v>38848.5</v>
@@ -2844,7 +2844,7 @@
         <v>1</v>
       </c>
       <c r="K11" t="n">
-        <v>26.06</v>
+        <v>2.7</v>
       </c>
       <c r="L11" t="n">
         <v>53910</v>
@@ -2885,7 +2885,7 @@
         <v>1</v>
       </c>
       <c r="K12" t="n">
-        <v>37.08</v>
+        <v>5.56</v>
       </c>
       <c r="L12" t="n">
         <v>91770</v>
@@ -2926,7 +2926,7 @@
         <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>29.43</v>
+        <v>4.75</v>
       </c>
       <c r="L13" t="n">
         <v>71700</v>
@@ -2967,7 +2967,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>22.36</v>
+        <v>0.97</v>
       </c>
       <c r="L14" t="n">
         <v>33900</v>
@@ -3008,7 +3008,7 @@
         <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>8.869999999999999</v>
+        <v>0</v>
       </c>
       <c r="L15" t="n">
         <v>14520</v>
@@ -3049,7 +3049,7 @@
         <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
         <v>7500</v>
@@ -3090,7 +3090,7 @@
         <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L17" t="n">
         <v>1860</v>
@@ -3131,7 +3131,7 @@
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
         <v>3810</v>
@@ -3602,7 +3602,7 @@
         <v>21850.2</v>
       </c>
       <c r="K5" t="n">
-        <v>96432.22</v>
+        <v>48216.11</v>
       </c>
       <c r="L5" t="n">
         <v>771120</v>
@@ -3643,7 +3643,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>492357.84</v>
+        <v>221561.03</v>
       </c>
       <c r="L6" t="n">
         <v>1418580</v>
@@ -3684,7 +3684,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>619574.5600000001</v>
+        <v>309787.28</v>
       </c>
       <c r="L7" t="n">
         <v>2860920</v>
@@ -3725,7 +3725,7 @@
         <v>20636.3</v>
       </c>
       <c r="K8" t="n">
-        <v>643269.89</v>
+        <v>393109.38</v>
       </c>
       <c r="L8" t="n">
         <v>4708152</v>
@@ -3766,7 +3766,7 @@
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>1091733.1</v>
+        <v>389904.68</v>
       </c>
       <c r="L9" t="n">
         <v>6714090</v>
@@ -3807,7 +3807,7 @@
         <v>121390</v>
       </c>
       <c r="K10" t="n">
-        <v>718143.24</v>
+        <v>84487.44</v>
       </c>
       <c r="L10" t="n">
         <v>6992730</v>
@@ -3848,7 +3848,7 @@
         <v>24278</v>
       </c>
       <c r="K11" t="n">
-        <v>1265199.41</v>
+        <v>130882.7</v>
       </c>
       <c r="L11" t="n">
         <v>9703800</v>
@@ -3889,7 +3889,7 @@
         <v>24278</v>
       </c>
       <c r="K12" t="n">
-        <v>1800456.48</v>
+        <v>270068.47</v>
       </c>
       <c r="L12" t="n">
         <v>16518600</v>
@@ -3930,7 +3930,7 @@
         <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>1429221.58</v>
+        <v>230519.61</v>
       </c>
       <c r="L13" t="n">
         <v>12906000</v>
@@ -3971,7 +3971,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>1085517.94</v>
+        <v>47196.43</v>
       </c>
       <c r="L14" t="n">
         <v>6102000</v>
@@ -4012,7 +4012,7 @@
         <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>430885.94</v>
+        <v>0</v>
       </c>
       <c r="L15" t="n">
         <v>2613600</v>
@@ -4053,7 +4053,7 @@
         <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>145668</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
         <v>1350000</v>
@@ -4094,7 +4094,7 @@
         <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>48556</v>
+        <v>0</v>
       </c>
       <c r="L17" t="n">
         <v>334800</v>
@@ -4135,7 +4135,7 @@
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>48556</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
         <v>685800</v>
@@ -4565,7 +4565,7 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>64</v>
+        <v>40</v>
       </c>
       <c r="L4" t="n">
         <v>145890</v>
@@ -4606,7 +4606,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="L5" t="n">
         <v>58680</v>
@@ -4647,7 +4647,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L6" t="n">
         <v>11220</v>
@@ -5610,7 +5610,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>9.6</v>
+        <v>4.96</v>
       </c>
       <c r="L5" t="n">
         <v>12322.8</v>
@@ -5651,7 +5651,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>0.51</v>
+        <v>0</v>
       </c>
       <c r="L6" t="n">
         <v>4151.4</v>
@@ -6614,7 +6614,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>466089.04</v>
+        <v>241080.54</v>
       </c>
       <c r="L5" t="n">
         <v>2218104</v>
@@ -6655,7 +6655,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>24617.89</v>
+        <v>0</v>
       </c>
       <c r="L6" t="n">
         <v>747252</v>
@@ -7577,7 +7577,7 @@
         <v>10</v>
       </c>
       <c r="K4" t="n">
-        <v>175</v>
+        <v>37</v>
       </c>
       <c r="L4" t="n">
         <v>138300</v>
@@ -7618,7 +7618,7 @@
         <v>1</v>
       </c>
       <c r="K5" t="n">
-        <v>48</v>
+        <v>11</v>
       </c>
       <c r="L5" t="n">
         <v>48690</v>
@@ -7659,7 +7659,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="L6" t="n">
         <v>13890</v>
@@ -7700,7 +7700,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L7" t="n">
         <v>3780</v>
@@ -7741,7 +7741,7 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L8" t="n">
         <v>2040</v>
@@ -8622,7 +8622,7 @@
         <v>0.3</v>
       </c>
       <c r="K5" t="n">
-        <v>15.89</v>
+        <v>3.64</v>
       </c>
       <c r="L5" t="n">
         <v>10224.9</v>
@@ -8663,7 +8663,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>4.56</v>
+        <v>0</v>
       </c>
       <c r="L6" t="n">
         <v>5139.3</v>
@@ -8704,7 +8704,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>1.28</v>
+        <v>0</v>
       </c>
       <c r="L7" t="n">
         <v>2268</v>
@@ -8745,7 +8745,7 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>1.47</v>
+        <v>0</v>
       </c>
       <c r="L8" t="n">
         <v>1448.4</v>
@@ -9626,7 +9626,7 @@
         <v>7283.4</v>
       </c>
       <c r="K5" t="n">
-        <v>771457.73</v>
+        <v>176792.4</v>
       </c>
       <c r="L5" t="n">
         <v>1840482</v>
@@ -9667,7 +9667,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="n">
-        <v>221561.03</v>
+        <v>0</v>
       </c>
       <c r="L6" t="n">
         <v>925074</v>
@@ -9708,7 +9708,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>61957.46</v>
+        <v>0</v>
       </c>
       <c r="L7" t="n">
         <v>408240</v>
@@ -9749,7 +9749,7 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>71474.42999999999</v>
+        <v>0</v>
       </c>
       <c r="L8" t="n">
         <v>260712</v>
@@ -10589,7 +10589,7 @@
         <v>9</v>
       </c>
       <c r="K4" t="n">
-        <v>229</v>
+        <v>131</v>
       </c>
       <c r="L4" t="n">
         <v>172410</v>
@@ -10630,7 +10630,7 @@
         <v>10</v>
       </c>
       <c r="K5" t="n">
-        <v>161</v>
+        <v>88</v>
       </c>
       <c r="L5" t="n">
         <v>162240</v>
@@ -10671,7 +10671,7 @@
         <v>6</v>
       </c>
       <c r="K6" t="n">
-        <v>151</v>
+        <v>76</v>
       </c>
       <c r="L6" t="n">
         <v>156300</v>
@@ -10712,7 +10712,7 @@
         <v>1</v>
       </c>
       <c r="K7" t="n">
-        <v>204</v>
+        <v>72</v>
       </c>
       <c r="L7" t="n">
         <v>202470</v>
@@ -10753,7 +10753,7 @@
         <v>2</v>
       </c>
       <c r="K8" t="n">
-        <v>125</v>
+        <v>42</v>
       </c>
       <c r="L8" t="n">
         <v>127230</v>
@@ -10794,7 +10794,7 @@
         <v>1</v>
       </c>
       <c r="K9" t="n">
-        <v>92</v>
+        <v>34</v>
       </c>
       <c r="L9" t="n">
         <v>74640</v>
@@ -10835,7 +10835,7 @@
         <v>2</v>
       </c>
       <c r="K10" t="n">
-        <v>46</v>
+        <v>5</v>
       </c>
       <c r="L10" t="n">
         <v>39240</v>
@@ -10876,7 +10876,7 @@
         <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L11" t="n">
         <v>10200</v>
@@ -11163,7 +11163,7 @@
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
         <v>600</v>
@@ -11634,7 +11634,7 @@
         <v>7.5</v>
       </c>
       <c r="K5" t="n">
-        <v>200.92</v>
+        <v>86.72</v>
       </c>
       <c r="L5" t="n">
         <v>186612.3</v>
@@ -11675,7 +11675,7 @@
         <v>6.5</v>
       </c>
       <c r="K6" t="n">
-        <v>215.98</v>
+        <v>83.66</v>
       </c>
       <c r="L6" t="n">
         <v>212809.2</v>
@@ -11716,7 +11716,7 @@
         <v>7.7</v>
       </c>
       <c r="K7" t="n">
-        <v>285.19</v>
+        <v>96.98</v>
       </c>
       <c r="L7" t="n">
         <v>320040</v>
@@ -11757,7 +11757,7 @@
         <v>8.5</v>
       </c>
       <c r="K8" t="n">
-        <v>261.28</v>
+        <v>75.06999999999999</v>
       </c>
       <c r="L8" t="n">
         <v>313962</v>
@@ -11798,7 +11798,7 @@
         <v>3.8</v>
       </c>
       <c r="K9" t="n">
-        <v>274.63</v>
+        <v>88.33</v>
       </c>
       <c r="L9" t="n">
         <v>305183.7</v>
@@ -11839,7 +11839,7 @@
         <v>11</v>
       </c>
       <c r="K10" t="n">
-        <v>221.85</v>
+        <v>51.33</v>
       </c>
       <c r="L10" t="n">
         <v>266519.4</v>
@@ -11880,7 +11880,7 @@
         <v>3</v>
       </c>
       <c r="K11" t="n">
-        <v>155.44</v>
+        <v>31.45</v>
       </c>
       <c r="L11" t="n">
         <v>187320</v>
@@ -11921,7 +11921,7 @@
         <v>2</v>
       </c>
       <c r="K12" t="n">
-        <v>105.68</v>
+        <v>15.76</v>
       </c>
       <c r="L12" t="n">
         <v>151590</v>
@@ -11962,7 +11962,7 @@
         <v>3</v>
       </c>
       <c r="K13" t="n">
-        <v>53.17</v>
+        <v>5.7</v>
       </c>
       <c r="L13" t="n">
         <v>102240</v>
@@ -12003,7 +12003,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>32.08</v>
+        <v>0.97</v>
       </c>
       <c r="L14" t="n">
         <v>43560</v>
@@ -12044,7 +12044,7 @@
         <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>8.869999999999999</v>
+        <v>0</v>
       </c>
       <c r="L15" t="n">
         <v>18390</v>
@@ -12085,7 +12085,7 @@
         <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
         <v>8700</v>
@@ -12126,7 +12126,7 @@
         <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L17" t="n">
         <v>2460</v>
@@ -12167,7 +12167,7 @@
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
         <v>4620</v>
@@ -12638,7 +12638,7 @@
         <v>3</v>
       </c>
       <c r="K5" t="n">
-        <v>53.29</v>
+        <v>29.13</v>
       </c>
       <c r="L5" t="n">
         <v>34070.4</v>
@@ -12679,7 +12679,7 @@
         <v>3</v>
       </c>
       <c r="K6" t="n">
-        <v>76.56</v>
+        <v>38.53</v>
       </c>
       <c r="L6" t="n">
         <v>57831</v>
@@ -12720,7 +12720,7 @@
         <v>0.7</v>
       </c>
       <c r="K7" t="n">
-        <v>130.15</v>
+        <v>45.94</v>
       </c>
       <c r="L7" t="n">
         <v>121482</v>
@@ -12761,7 +12761,7 @@
         <v>1.7</v>
       </c>
       <c r="K8" t="n">
-        <v>92</v>
+        <v>30.91</v>
       </c>
       <c r="L8" t="n">
         <v>90333.3</v>
@@ -12802,7 +12802,7 @@
         <v>0.95</v>
       </c>
       <c r="K9" t="n">
-        <v>73.88</v>
+        <v>27.3</v>
       </c>
       <c r="L9" t="n">
         <v>60458.4</v>
@@ -12843,7 +12843,7 @@
         <v>2</v>
       </c>
       <c r="K10" t="n">
-        <v>40.02</v>
+        <v>4.35</v>
       </c>
       <c r="L10" t="n">
         <v>34923.6</v>
@@ -12884,7 +12884,7 @@
         <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>4.49</v>
+        <v>1.8</v>
       </c>
       <c r="L11" t="n">
         <v>10200</v>
@@ -13171,7 +13171,7 @@
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
         <v>600</v>
@@ -13642,7 +13642,7 @@
         <v>72834</v>
       </c>
       <c r="K5" t="n">
-        <v>2587597.8</v>
+        <v>1414339.17</v>
       </c>
       <c r="L5" t="n">
         <v>6132672</v>
@@ -13683,7 +13683,7 @@
         <v>72834</v>
       </c>
       <c r="K6" t="n">
-        <v>3717301.69</v>
+        <v>1870959.79</v>
       </c>
       <c r="L6" t="n">
         <v>10409580</v>
@@ -13724,7 +13724,7 @@
         <v>16994.6</v>
       </c>
       <c r="K7" t="n">
-        <v>6319660.51</v>
+        <v>2230468.42</v>
       </c>
       <c r="L7" t="n">
         <v>21866760</v>
@@ -13765,7 +13765,7 @@
         <v>41272.6</v>
       </c>
       <c r="K8" t="n">
-        <v>4467152</v>
+        <v>1500963.07</v>
       </c>
       <c r="L8" t="n">
         <v>16259994</v>
@@ -13806,7 +13806,7 @@
         <v>23064.1</v>
       </c>
       <c r="K9" t="n">
-        <v>3587123.06</v>
+        <v>1325675.91</v>
       </c>
       <c r="L9" t="n">
         <v>10882512</v>
@@ -13847,7 +13847,7 @@
         <v>48556</v>
       </c>
       <c r="K10" t="n">
-        <v>1943211.12</v>
+        <v>211218.6</v>
       </c>
       <c r="L10" t="n">
         <v>6286248</v>
@@ -13888,7 +13888,7 @@
         <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>218137.83</v>
+        <v>87255.13</v>
       </c>
       <c r="L11" t="n">
         <v>1836000</v>
@@ -14175,7 +14175,7 @@
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>48556</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
         <v>108000</v>
@@ -14605,7 +14605,7 @@
         <v>4</v>
       </c>
       <c r="K4" t="n">
-        <v>118</v>
+        <v>48</v>
       </c>
       <c r="L4" t="n">
         <v>345870</v>
@@ -14646,7 +14646,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="L5" t="n">
         <v>112080</v>
@@ -15650,7 +15650,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>10.59</v>
+        <v>4.96</v>
       </c>
       <c r="L5" t="n">
         <v>23536.8</v>
@@ -16654,7 +16654,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>514305.15</v>
+        <v>241080.54</v>
       </c>
       <c r="L5" t="n">
         <v>4236624</v>
@@ -17658,7 +17658,7 @@
         <v>182085</v>
       </c>
       <c r="K5" t="n">
-        <v>9755725.85</v>
+        <v>4210873.43</v>
       </c>
       <c r="L5" t="n">
         <v>33590214</v>
@@ -17699,7 +17699,7 @@
         <v>157807</v>
       </c>
       <c r="K6" t="n">
-        <v>10487221.99</v>
+        <v>4061952.18</v>
       </c>
       <c r="L6" t="n">
         <v>38305656</v>
@@ -17740,7 +17740,7 @@
         <v>186940.6</v>
       </c>
       <c r="K7" t="n">
-        <v>13847491.42</v>
+        <v>4708766.66</v>
       </c>
       <c r="L7" t="n">
         <v>57607200</v>
@@ -17781,7 +17781,7 @@
         <v>206363</v>
       </c>
       <c r="K8" t="n">
-        <v>12686711.68</v>
+        <v>3645196.03</v>
       </c>
       <c r="L8" t="n">
         <v>56513160</v>
@@ -17822,7 +17822,7 @@
         <v>92256.39999999999</v>
       </c>
       <c r="K9" t="n">
-        <v>13334740.06</v>
+        <v>4288951.48</v>
       </c>
       <c r="L9" t="n">
         <v>54933066</v>
@@ -17863,7 +17863,7 @@
         <v>267058</v>
       </c>
       <c r="K10" t="n">
-        <v>10772148.6</v>
+        <v>2492379.48</v>
       </c>
       <c r="L10" t="n">
         <v>47973492</v>
@@ -17904,7 +17904,7 @@
         <v>72834</v>
       </c>
       <c r="K11" t="n">
-        <v>7547568.92</v>
+        <v>1526964.81</v>
       </c>
       <c r="L11" t="n">
         <v>33717600</v>
@@ -17945,7 +17945,7 @@
         <v>48556</v>
       </c>
       <c r="K12" t="n">
-        <v>5131300.97</v>
+        <v>765194</v>
       </c>
       <c r="L12" t="n">
         <v>27286200</v>
@@ -17986,7 +17986,7 @@
         <v>72834</v>
       </c>
       <c r="K13" t="n">
-        <v>2581819.63</v>
+        <v>276623.53</v>
       </c>
       <c r="L13" t="n">
         <v>18403200</v>
@@ -18027,7 +18027,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>1557482.26</v>
+        <v>47196.43</v>
       </c>
       <c r="L14" t="n">
         <v>7840800</v>
@@ -18068,7 +18068,7 @@
         <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>430885.94</v>
+        <v>0</v>
       </c>
       <c r="L15" t="n">
         <v>3310200</v>
@@ -18109,7 +18109,7 @@
         <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>194224</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
         <v>1566000</v>
@@ -18150,7 +18150,7 @@
         <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>97112</v>
+        <v>0</v>
       </c>
       <c r="L17" t="n">
         <v>442800</v>
@@ -18191,7 +18191,7 @@
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>97112</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
         <v>831600</v>
@@ -18621,7 +18621,7 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>122</v>
+        <v>72</v>
       </c>
       <c r="L4" t="n">
         <v>135660</v>
@@ -18662,7 +18662,7 @@
         <v>2</v>
       </c>
       <c r="K5" t="n">
-        <v>139</v>
+        <v>69</v>
       </c>
       <c r="L5" t="n">
         <v>165450</v>
@@ -18703,7 +18703,7 @@
         <v>4</v>
       </c>
       <c r="K6" t="n">
-        <v>136</v>
+        <v>53</v>
       </c>
       <c r="L6" t="n">
         <v>168420</v>
@@ -18744,7 +18744,7 @@
         <v>7</v>
       </c>
       <c r="K7" t="n">
-        <v>144</v>
+        <v>57</v>
       </c>
       <c r="L7" t="n">
         <v>179910</v>
@@ -18785,7 +18785,7 @@
         <v>7</v>
       </c>
       <c r="K8" t="n">
-        <v>201</v>
+        <v>48</v>
       </c>
       <c r="L8" t="n">
         <v>236760</v>
@@ -18826,7 +18826,7 @@
         <v>3</v>
       </c>
       <c r="K9" t="n">
-        <v>219</v>
+        <v>65</v>
       </c>
       <c r="L9" t="n">
         <v>238920</v>
@@ -18867,7 +18867,7 @@
         <v>4</v>
       </c>
       <c r="K10" t="n">
-        <v>192</v>
+        <v>52</v>
       </c>
       <c r="L10" t="n">
         <v>208200</v>
@@ -18908,7 +18908,7 @@
         <v>2</v>
       </c>
       <c r="K11" t="n">
-        <v>139</v>
+        <v>30</v>
       </c>
       <c r="L11" t="n">
         <v>121080</v>
@@ -18949,7 +18949,7 @@
         <v>1</v>
       </c>
       <c r="K12" t="n">
-        <v>72</v>
+        <v>9</v>
       </c>
       <c r="L12" t="n">
         <v>54450</v>
@@ -18990,7 +18990,7 @@
         <v>3</v>
       </c>
       <c r="K13" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="L13" t="n">
         <v>27270</v>
@@ -19031,7 +19031,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L14" t="n">
         <v>8070</v>
@@ -19113,7 +19113,7 @@
         <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
         <v>960</v>
@@ -19154,7 +19154,7 @@
         <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L17" t="n">
         <v>210</v>
@@ -19666,7 +19666,7 @@
         <v>0.6</v>
       </c>
       <c r="K5" t="n">
-        <v>46.01</v>
+        <v>22.84</v>
       </c>
       <c r="L5" t="n">
         <v>34744.5</v>
@@ -19707,7 +19707,7 @@
         <v>2</v>
       </c>
       <c r="K6" t="n">
-        <v>68.95</v>
+        <v>26.87</v>
       </c>
       <c r="L6" t="n">
         <v>62315.4</v>
@@ -19748,7 +19748,7 @@
         <v>4.9</v>
       </c>
       <c r="K7" t="n">
-        <v>91.87</v>
+        <v>36.37</v>
       </c>
       <c r="L7" t="n">
         <v>107946</v>
@@ -19789,7 +19789,7 @@
         <v>5.95</v>
       </c>
       <c r="K8" t="n">
-        <v>147.94</v>
+        <v>35.33</v>
       </c>
       <c r="L8" t="n">
         <v>168099.6</v>
@@ -19830,7 +19830,7 @@
         <v>2.85</v>
       </c>
       <c r="K9" t="n">
-        <v>175.86</v>
+        <v>52.2</v>
       </c>
       <c r="L9" t="n">
         <v>193525.2</v>
@@ -19871,7 +19871,7 @@
         <v>4</v>
       </c>
       <c r="K10" t="n">
-        <v>167.04</v>
+        <v>45.24</v>
       </c>
       <c r="L10" t="n">
         <v>185298</v>
@@ -19912,7 +19912,7 @@
         <v>2</v>
       </c>
       <c r="K11" t="n">
-        <v>124.89</v>
+        <v>26.96</v>
       </c>
       <c r="L11" t="n">
         <v>121080</v>
@@ -19953,7 +19953,7 @@
         <v>1</v>
       </c>
       <c r="K12" t="n">
-        <v>66.73999999999999</v>
+        <v>8.34</v>
       </c>
       <c r="L12" t="n">
         <v>54450</v>
@@ -19994,7 +19994,7 @@
         <v>3</v>
       </c>
       <c r="K13" t="n">
-        <v>23.74</v>
+        <v>0.95</v>
       </c>
       <c r="L13" t="n">
         <v>27270</v>
@@ -20035,7 +20035,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>9.720000000000001</v>
+        <v>0</v>
       </c>
       <c r="L14" t="n">
         <v>8070</v>
@@ -20117,7 +20117,7 @@
         <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
         <v>960</v>
@@ -20158,7 +20158,7 @@
         <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L17" t="n">
         <v>210</v>
@@ -20670,7 +20670,7 @@
         <v>14566.8</v>
       </c>
       <c r="K5" t="n">
-        <v>2234013</v>
+        <v>1108970.48</v>
       </c>
       <c r="L5" t="n">
         <v>6254010</v>
@@ -20711,7 +20711,7 @@
         <v>48556</v>
       </c>
       <c r="K6" t="n">
-        <v>3348033.31</v>
+        <v>1304748.28</v>
       </c>
       <c r="L6" t="n">
         <v>11216772</v>
@@ -20752,7 +20752,7 @@
         <v>118962.2</v>
       </c>
       <c r="K7" t="n">
-        <v>4460936.83</v>
+        <v>1765787.5</v>
       </c>
       <c r="L7" t="n">
         <v>19430280</v>
@@ -20793,7 +20793,7 @@
         <v>144454.1</v>
       </c>
       <c r="K8" t="n">
-        <v>7183180.42</v>
+        <v>1715386.37</v>
       </c>
       <c r="L8" t="n">
         <v>30257928</v>
@@ -20834,7 +20834,7 @@
         <v>69192.3</v>
       </c>
       <c r="K9" t="n">
-        <v>8538912.49</v>
+        <v>2534380.42</v>
       </c>
       <c r="L9" t="n">
         <v>34834536</v>
@@ -20875,7 +20875,7 @@
         <v>97112</v>
       </c>
       <c r="K10" t="n">
-        <v>8110794.24</v>
+        <v>2196673.44</v>
       </c>
       <c r="L10" t="n">
         <v>33353640</v>
@@ -20916,7 +20916,7 @@
         <v>48556</v>
       </c>
       <c r="K11" t="n">
-        <v>6064231.67</v>
+        <v>1308826.98</v>
       </c>
       <c r="L11" t="n">
         <v>21794400</v>
@@ -20957,7 +20957,7 @@
         <v>24278</v>
       </c>
       <c r="K12" t="n">
-        <v>3240821.66</v>
+        <v>405102.71</v>
       </c>
       <c r="L12" t="n">
         <v>9801000</v>
@@ -20998,7 +20998,7 @@
         <v>72834</v>
       </c>
       <c r="K13" t="n">
-        <v>1152598.05</v>
+        <v>46103.92</v>
       </c>
       <c r="L13" t="n">
         <v>4908600</v>
@@ -21039,7 +21039,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>471964.32</v>
+        <v>0</v>
       </c>
       <c r="L14" t="n">
         <v>1452600</v>
@@ -21121,7 +21121,7 @@
         <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>48556</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
         <v>172800</v>
@@ -21162,7 +21162,7 @@
         <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>48556</v>
+        <v>0</v>
       </c>
       <c r="L17" t="n">
         <v>37800</v>
@@ -21633,7 +21633,7 @@
         <v>14</v>
       </c>
       <c r="K4" t="n">
-        <v>388</v>
+        <v>96</v>
       </c>
       <c r="L4" t="n">
         <v>407070</v>
@@ -21674,7 +21674,7 @@
         <v>7</v>
       </c>
       <c r="K5" t="n">
-        <v>191</v>
+        <v>61</v>
       </c>
       <c r="L5" t="n">
         <v>261780</v>
@@ -21715,7 +21715,7 @@
         <v>3</v>
       </c>
       <c r="K6" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="L6" t="n">
         <v>135120</v>
@@ -21756,7 +21756,7 @@
         <v>3</v>
       </c>
       <c r="K7" t="n">
-        <v>74</v>
+        <v>12</v>
       </c>
       <c r="L7" t="n">
         <v>79380</v>
@@ -21797,7 +21797,7 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="L8" t="n">
         <v>21930</v>
@@ -22678,7 +22678,7 @@
         <v>2.1</v>
       </c>
       <c r="K5" t="n">
-        <v>63.22</v>
+        <v>20.19</v>
       </c>
       <c r="L5" t="n">
         <v>54973.8</v>
@@ -22719,7 +22719,7 @@
         <v>1.5</v>
       </c>
       <c r="K6" t="n">
-        <v>54.76</v>
+        <v>13.69</v>
       </c>
       <c r="L6" t="n">
         <v>49994.4</v>
@@ -22760,7 +22760,7 @@
         <v>2.1</v>
       </c>
       <c r="K7" t="n">
-        <v>47.21</v>
+        <v>7.66</v>
       </c>
       <c r="L7" t="n">
         <v>47628</v>
@@ -22801,7 +22801,7 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>6.62</v>
+        <v>0.74</v>
       </c>
       <c r="L8" t="n">
         <v>15570.3</v>
@@ -23682,7 +23682,7 @@
         <v>50983.8</v>
       </c>
       <c r="K5" t="n">
-        <v>3069758.88</v>
+        <v>980394.2</v>
       </c>
       <c r="L5" t="n">
         <v>9895284</v>
@@ -23723,7 +23723,7 @@
         <v>36417</v>
       </c>
       <c r="K6" t="n">
-        <v>2658732.34</v>
+        <v>664683.08</v>
       </c>
       <c r="L6" t="n">
         <v>8998992</v>
@@ -23764,7 +23764,7 @@
         <v>50983.8</v>
       </c>
       <c r="K7" t="n">
-        <v>2292425.87</v>
+        <v>371744.74</v>
       </c>
       <c r="L7" t="n">
         <v>8573040</v>
@@ -23805,7 +23805,7 @@
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>321634.94</v>
+        <v>35737.22</v>
       </c>
       <c r="L8" t="n">
         <v>2802654</v>

</xml_diff>